<commit_message>
update WCR dashboard data 2026-06-26 15:20
</commit_message>
<xml_diff>
--- a/docs/reports/WCR_Kavach_Unified_KPI_Jun15-Jun21.xlsx
+++ b/docs/reports/WCR_Kavach_Unified_KPI_Jun15-Jun21.xlsx
@@ -709,7 +709,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Period: 15 Jun - 21 Jun 2026  ·  all locomotives  ·  one combined row</t>
+          <t>Period: Jun15 - Jun21 (custom)  ·  all locomotives  ·  one combined row</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>15 Jun - 21 Jun 2026</t>
+          <t>Jun15 - Jun21 (custom)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -11590,7 +11590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11609,6 +11609,9 @@
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="46" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11708,8 +11711,23 @@
           <t>Suspected Reason (undesirable)</t>
         </is>
       </c>
-    </row>
-    <row r="6">
+      <c r="Q5" s="14" t="inlineStr">
+        <is>
+          <t>Points/Track condition</t>
+        </is>
+      </c>
+      <c r="R5" s="14" t="inlineStr">
+        <is>
+          <t>Signal Aspect Analysis</t>
+        </is>
+      </c>
+      <c r="S5" s="14" t="inlineStr">
+        <is>
+          <t>Loco Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="289" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
         <is>
           <t>16 Jun</t>
@@ -11782,8 +11800,26 @@
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="7">
+      <c r="Q6" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit SV28.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 138 m short of SV28 (sig abs 918828); EB onset 14:49:24 at 55 km/h @ abs 918966 (138 m before SV28); halt 14:50:00 @ abs 918801 (27 m past SV28).</t>
+        </is>
+      </c>
+      <c r="R6" s="33" t="inlineStr">
+        <is>
+          <t>• At 14:49:03:240, the approach signal SV28 was displaying BLANK (BLANK) in the field but YELLOW (Y) on the DMI — a field/DMI aspect mismatch.
+• At 14:49:08 on 16/06/2026, the approach signal SV28 showed RED (R) in the field / RED (R) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S6" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="274" customHeight="1">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>16 Jun</t>
@@ -11843,7 +11879,7 @@
       </c>
       <c r="N7" s="33" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O7" s="31" t="inlineStr">
@@ -11856,8 +11892,26 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-    </row>
-    <row r="8">
+      <c r="Q7" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit S2.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 950 m short of S2 (sig abs 917851); EB onset 14:51:28 at 0 km/h @ abs 918801 (950 m before S2); halt 14:51:28 @ abs 918801 (950 m before S2).</t>
+        </is>
+      </c>
+      <c r="R7" s="33" t="inlineStr">
+        <is>
+          <t>• At 14:40:15:583, the approach signal S2 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.
+• At 14:49:50 on 16/06/2026, the approach signal S2 showed GREEN (G) in the field / GREEN (G) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S7" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="289" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>16 Jun</t>
@@ -11930,8 +11984,26 @@
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="9">
+      <c r="Q8" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit SV28.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 119 m short of SV28 (sig abs 918828); EB onset 18:29:06 at 52 km/h @ abs 918947 (119 m before SV28); halt 18:29:30 @ abs 918821 (7 m past SV28).</t>
+        </is>
+      </c>
+      <c r="R8" s="33" t="inlineStr">
+        <is>
+          <t>• At 18:28:49:436, the approach signal SV28 was displaying BLANK (BLANK) in the field but YELLOW (Y) on the DMI — a field/DMI aspect mismatch.
+• At 18:28:55 on 16/06/2026, the approach signal SV28 showed RED (R) in the field / RED (R) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S8" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="439" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>16 Jun</t>
@@ -12004,8 +12076,27 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-    </row>
-    <row r="10">
+      <c r="Q9" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry S28 → exit S2 (EntrySigId 9 / ExitSigId 11).
+Condition: route clear — points P231/232, P225/226, P223/224, P221/222, P217/218, P209/210 (favourable/free).
+FIU contacts: point P231/232 (c94) P→favourable; point P225/226 (c90) P→favourable; point P223/224 (c88) P→favourable; point P221/222 (c86) P→favourable; point P217/218 (c84) P→favourable; point P209/210 (c80) P→favourable.
+Loco: loco 970 m short of S2 (sig abs 917851); EB onset 18:30:36 at 0 km/h @ abs 918821 (970 m before S2); halt 18:30:36 @ abs 918821 (970 m before S2).</t>
+        </is>
+      </c>
+      <c r="R9" s="33" t="inlineStr">
+        <is>
+          <t>• At 18:02:13:699, the ahead signal S2 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.
+• At 18:29:22:330, the approach signal S28 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.</t>
+        </is>
+      </c>
+      <c r="S9" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="439" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>16 Jun</t>
@@ -12065,7 +12156,7 @@
       </c>
       <c r="N10" s="33" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>0</t>
         </is>
       </c>
       <c r="O10" s="31" t="inlineStr">
@@ -12078,8 +12169,27 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="49" customHeight="1">
+      <c r="Q10" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry S28 → exit S2 (EntrySigId 9 / ExitSigId 11).
+Condition: route clear — points P231/232, P225/226, P223/224, P221/222, P217/218, P209/210 (favourable/free).
+FIU contacts: point P231/232 (c94) P→favourable; point P225/226 (c90) P→favourable; point P223/224 (c88) P→favourable; point P221/222 (c86) P→favourable; point P217/218 (c84) P→favourable; point P209/210 (c80) P→favourable.
+Loco: loco 970 m short of S2 (sig abs 917851); EB onset 18:31:24 at 0 km/h @ abs 918821 (970 m before S2); halt 18:31:26 @ abs 918821 (970 m before S2).</t>
+        </is>
+      </c>
+      <c r="R10" s="33" t="inlineStr">
+        <is>
+          <t>• At 18:02:13:699, the ahead signal S2 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.
+• At 18:29:22:330, the approach signal S28 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.</t>
+        </is>
+      </c>
+      <c r="S10" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="439" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>17 Jun</t>
@@ -12153,8 +12263,26 @@
           <t>PG issue (speed fluctuation); Trip mode</t>
         </is>
       </c>
-    </row>
-    <row r="12">
+      <c r="Q11" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry S28 → exit S2 (EntrySigId 9 / ExitSigId 11).
+Condition: route clear — points P231/232, P225/226, P223/224, P221/222, P217/218, P209/210 (favourable/free).
+FIU contacts: point P231/232 (c94) P→favourable; point P225/226 (c90) P→favourable; point P223/224 (c88) P→favourable; point P221/222 (c86) P→favourable; point P217/218 (c84) P→favourable; point P209/210 (c80) P→favourable.
+Loco: loco 973 m short of S2 (sig abs 917851); EB onset 00:01:20 at 4 km/h @ abs 918824 (973 m before S2); halt 00:01:56 @ abs 918824 (973 m before S2).</t>
+        </is>
+      </c>
+      <c r="R11" s="33" t="inlineStr">
+        <is>
+          <t>@ 00:00:04 on 17/06/2026: S28 (col 9): field GREEN (G), DMI GREEN (G); S2 (col 11): field GREEN (G), DMI GREEN (G)</t>
+        </is>
+      </c>
+      <c r="S11" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="439" customHeight="1">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>17 Jun</t>
@@ -12227,8 +12355,26 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-    </row>
-    <row r="13">
+      <c r="Q12" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry S28 → exit S2 (EntrySigId 9 / ExitSigId 11).
+Condition: route clear — points P231/232, P225/226, P223/224, P221/222, P217/218, P209/210 (favourable/free).
+FIU contacts: point P231/232 (c94) P→favourable; point P225/226 (c90) P→favourable; point P223/224 (c88) P→favourable; point P221/222 (c86) P→favourable; point P217/218 (c84) P→favourable; point P209/210 (c80) P→favourable.
+Loco: loco 973 m short of S2 (sig abs 917851); EB onset 00:03:10 at 0 km/h @ abs 918824 (973 m before S2); halt 00:03:10 @ abs 918824 (973 m before S2).</t>
+        </is>
+      </c>
+      <c r="R12" s="33" t="inlineStr">
+        <is>
+          <t>• At 00:01:21:551, the approach signal S28 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.</t>
+        </is>
+      </c>
+      <c r="S12" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="229" customHeight="1">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>18 Jun</t>
@@ -12301,8 +12447,25 @@
           <t>EB at 0-1 km/h; Shunting mode</t>
         </is>
       </c>
-    </row>
-    <row r="14">
+      <c r="Q13" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit S44.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 869 m short of S44 (sig abs 1028164); EB onset 02:15:04 at 0 km/h @ abs 1029033 (869 m before S44); halt 02:16:34 @ abs 1029033 (869 m before S44).</t>
+        </is>
+      </c>
+      <c r="R13" s="33" t="inlineStr">
+        <is>
+          <t>• At 02:14:31 on 18/06/2026, the approach signal S44 showed RED (R) in the field / RED (R) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S13" s="31" t="inlineStr">
+        <is>
+          <t>HBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="304" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>19 Jun</t>
@@ -12375,8 +12538,26 @@
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="15">
+      <c r="Q14" s="36" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit UPGATEINNDIST.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 1253 m short of UPGATEINNDIST (sig abs 1167280); EB onset 06:42:00 at 77 km/h @ abs 1166027 (1253 m before UPGATEINNDIST); halt 06:42:00 @ abs 1166027 (1253 m before UPGATEINNDIST).</t>
+        </is>
+      </c>
+      <c r="R14" s="36" t="inlineStr">
+        <is>
+          <t>• At 06:09:41:425, the approach signal UPGATEINNDIST was displaying GREEN (G) in the field but YELLOW (Y) on the DMI — a field/DMI aspect mismatch.
+• At 06:41:59 on 19/06/2026, the approach signal UPGATEINNDIST showed YELLOW (Y) in the field / YELLOW (Y) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S14" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="184" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
           <t>19 Jun</t>
@@ -12449,8 +12630,25 @@
           <t>FS-&gt;SR degradation + EB</t>
         </is>
       </c>
-    </row>
-    <row r="16">
+      <c r="Q15" s="36" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit SV28.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 1667 m short of SV28 (sig abs 918828); EB onset 11:04:08 at 21 km/h; halt 11:04:18.</t>
+        </is>
+      </c>
+      <c r="R15" s="36" t="inlineStr">
+        <is>
+          <t>• At 11:03:06 on 19/06/2026, the approach signal SV28 showed GREEN (G) in the field / GREEN (G) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S15" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="304" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>19 Jun</t>
@@ -12510,7 +12708,7 @@
       </c>
       <c r="N16" s="36" t="inlineStr">
         <is>
-          <t>5102</t>
+          <t>8087</t>
         </is>
       </c>
       <c r="O16" s="16" t="inlineStr">
@@ -12523,8 +12721,26 @@
           <t>Failure mode</t>
         </is>
       </c>
-    </row>
-    <row r="17">
+      <c r="Q16" s="36" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit DNIBSSIGS50.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 203 m short of DNIBSSIGS50 (sig abs 1206836); EB onset 11:18:54 at 128 km/h @ abs 1206633 (203 m before DNIBSSIGS50); halt 11:19:40 @ abs 1207504 (668 m past DNIBSSIGS50).</t>
+        </is>
+      </c>
+      <c r="R16" s="36" t="inlineStr">
+        <is>
+          <t>• At 10:19:58:159, the approach signal DNIBSSIGS50 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.
+• At 11:12:20 on 19/06/2026, the approach signal DNIBSSIGS50 showed GREEN (G) in the field / GREEN (G) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S16" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="274" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>19 Jun</t>
@@ -12597,8 +12813,26 @@
           <t>Failure mode</t>
         </is>
       </c>
-    </row>
-    <row r="18">
+      <c r="Q17" s="36" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit SF1.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 511 m short of SF1 (sig abs 1137765); EB onset 18:46:58 at 124 km/h @ abs 1138276 (511 m before SF1); halt 18:47:42 @ abs 1137483 (282 m past SF1).</t>
+        </is>
+      </c>
+      <c r="R17" s="36" t="inlineStr">
+        <is>
+          <t>• At 18:44:40:522, the approach signal SF1 was displaying GREEN (G) in the field but RED (R) on the DMI — a field/DMI aspect mismatch.
+• At 18:44:50 on 19/06/2026, the approach signal SF1 showed GREEN (G) in the field / GREEN (G) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S17" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>20 Jun</t>
@@ -12671,8 +12905,23 @@
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
+      <c r="Q18" s="33" t="inlineStr">
+        <is>
+          <t>n/a (ahead signal not resolved)</t>
+        </is>
+      </c>
+      <c r="R18" s="33" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="S18" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="229" customHeight="1">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>20 Jun</t>
@@ -12746,8 +12995,25 @@
           <t>Sudden MA drop; Failure mode</t>
         </is>
       </c>
-    </row>
-    <row r="20">
+      <c r="Q19" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit S12.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 494 m short of S12 (sig abs 963991); EB onset 15:45:16 at 128 km/h @ abs 964485 (494 m before S12); halt 15:46:26 @ abs 963486 (505 m past S12).</t>
+        </is>
+      </c>
+      <c r="R19" s="33" t="inlineStr">
+        <is>
+          <t>• At 15:44:50 on 20/06/2026, the approach signal S12 showed GREEN (G) in the field / GREEN (G) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S19" s="31" t="inlineStr">
+        <is>
+          <t>HBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="244" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>20 Jun</t>
@@ -12820,8 +13086,25 @@
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="21">
+      <c r="Q20" s="36" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit S45.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 1619 m short of S45 (sig abs 1028188); EB onset 21:11:08 at 33 km/h @ abs 1029807 (1619 m before S45); halt 21:11:22 @ abs 1029721 (1533 m before S45).</t>
+        </is>
+      </c>
+      <c r="R20" s="36" t="inlineStr">
+        <is>
+          <t>• At 21:10:43 on 20/06/2026, the approach signal S45 showed RED (R) in the field / RED (R) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S20" s="16" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="229" customHeight="1">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>21 Jun</t>
@@ -12894,8 +13177,25 @@
           <t>Trip mode</t>
         </is>
       </c>
-    </row>
-    <row r="22">
+      <c r="Q21" s="33" t="inlineStr">
+        <is>
+          <t>Route: entry ? → exit S46.
+Condition: no interlocked route resolved at this approach — points/tracks not determined.
+Loco: loco 774 m short of S46 (sig abs 1028199); EB onset 09:30:00 at 9 km/h @ abs 1028973 (774 m before S46); halt 09:31:12 @ abs 1028978 (779 m before S46).</t>
+        </is>
+      </c>
+      <c r="R21" s="33" t="inlineStr">
+        <is>
+          <t>• At 09:27:09 on 21/06/2026, the approach signal S46 showed RED (R) in the field / RED (R) on the DMI (field and DMI agree).</t>
+        </is>
+      </c>
+      <c r="S21" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>21 Jun</t>
@@ -12955,24 +13255,39 @@
       </c>
       <c r="N22" s="33" t="inlineStr">
         <is>
+          <t>7570</t>
+        </is>
+      </c>
+      <c r="O22" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" s="33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" s="33" t="inlineStr">
+        <is>
+          <t>n/a (ahead signal not resolved)</t>
+        </is>
+      </c>
+      <c r="R22" s="33" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="O22" s="31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P22" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="S22" s="31" t="inlineStr">
+        <is>
+          <t>Medha/Kernex</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A3:S3"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>